<commit_message>
Banco de dados 100% conectado e populado através de arquivo.
</commit_message>
<xml_diff>
--- a/src/Modelo Banco de Dados deskCatalog (1).xlsx
+++ b/src/Modelo Banco de Dados deskCatalog (1).xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29523"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="1145" documentId="11_7F4755BF84DCCE43E268565A8931F45BFA75341E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{356944BB-C198-4C0E-9B50-D2CB665FE087}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ritam\ProjetoVS Py\DeskCatalog\src\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A4DEEFD-AC93-4AD2-A7E7-9980B94F4678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -154,7 +159,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -601,30 +606,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.28515625" customWidth="1"/>
+    <col min="1" max="1" width="27.33203125" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" customWidth="1"/>
-    <col min="5" max="5" width="21.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" customWidth="1"/>
-    <col min="7" max="7" width="16.28515625" customWidth="1"/>
-    <col min="9" max="9" width="30.140625" customWidth="1"/>
-    <col min="10" max="10" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.44140625" customWidth="1"/>
+    <col min="5" max="5" width="21.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.6640625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="9" max="9" width="30.109375" customWidth="1"/>
+    <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="13" max="13" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="17" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="14" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="15.75" customHeight="1">
+    <row r="1" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -644,7 +649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -673,7 +678,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>7</v>
       </c>
@@ -702,7 +707,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -722,7 +727,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>16</v>
       </c>
@@ -742,7 +747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>4</v>
       </c>
@@ -771,7 +776,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
         <v>19</v>
       </c>
@@ -800,7 +805,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>23</v>
       </c>
@@ -829,7 +834,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>10</v>
       </c>
@@ -856,7 +861,7 @@
       </c>
       <c r="Y14" s="9"/>
     </row>
-    <row r="15" spans="1:25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>29</v>
       </c>
@@ -873,7 +878,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
       <c r="E16" t="s">
         <v>33</v>
       </c>
@@ -881,7 +886,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="5:6">
+    <row r="17" spans="5:6" x14ac:dyDescent="0.3">
       <c r="E17" t="s">
         <v>34</v>
       </c>
@@ -889,7 +894,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="5:6">
+    <row r="18" spans="5:6" x14ac:dyDescent="0.3">
       <c r="E18" t="s">
         <v>36</v>
       </c>
@@ -897,7 +902,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="5:6">
+    <row r="19" spans="5:6" x14ac:dyDescent="0.3">
       <c r="E19" s="10" t="s">
         <v>37</v>
       </c>
@@ -907,5 +912,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>